<commit_message>
umstrukturierung, Briefkopf fast fertig gestellt, Datenhandling überarbeitet
</commit_message>
<xml_diff>
--- a/data/zeiterfassung_januar.xlsx
+++ b/data/zeiterfassung_januar.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\silas\Desktop\rechnungsprogramm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\silas\Desktop\rechnungsprogramm\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02E40B0-89AB-4432-A4BA-E276FE21825A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95B4EDB9-D038-4F28-8F54-2113204D915F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="3135" windowWidth="29040" windowHeight="15720" xr2:uid="{A93BE20D-7F6F-4B8A-874D-CFF2A8466003}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t>Kunde:</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>KdNr.:</t>
+  </si>
+  <si>
+    <t>blaköjaldsgjöaoijf, öadfilgsaölfdgkbhaoidfbhölakdfjghäaoisjgaölsgkhjaöoeigknjöladsfg</t>
   </si>
 </sst>
 </file>
@@ -240,6 +243,30 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -248,30 +275,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -832,10 +835,10 @@
     <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="18"/>
       <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
@@ -844,24 +847,24 @@
       <c r="B4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="25">
+      <c r="C4" s="15">
         <v>1000</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="19"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="4">
         <v>45658</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="19"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="4">
         <v>45688</v>
       </c>
@@ -879,10 +882,10 @@
     <row r="9" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:6" s="7" customFormat="1" ht="38.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="22"/>
+      <c r="B11" s="19"/>
       <c r="C11" s="6" t="s">
         <v>5</v>
       </c>
@@ -897,10 +900,10 @@
       </c>
     </row>
     <row r="12" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="23">
+      <c r="A12" s="20">
         <v>45686</v>
       </c>
-      <c r="B12" s="24"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
@@ -916,133 +919,217 @@
       </c>
     </row>
     <row r="13" spans="1:6" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="20">
+      <c r="A13" s="22">
         <v>45688</v>
       </c>
-      <c r="B13" s="21"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="20"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="20"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="20"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="D13" s="11">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E13" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666669</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="22">
+        <v>45679</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="11">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="E14" s="11">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F14" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="22">
+        <v>45680</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="11">
+        <v>0.20833333333333301</v>
+      </c>
+      <c r="E15" s="11">
+        <v>0.375</v>
+      </c>
+      <c r="F15" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666699</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="22">
+        <v>45681</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="E16" s="11">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="F16" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666702</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="22">
+        <v>45682</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="11">
+        <v>0.29166666666666702</v>
+      </c>
+      <c r="E17" s="11">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="F17" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666596</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="22">
+        <v>45683</v>
+      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="11">
+        <v>0.33333333333333298</v>
+      </c>
+      <c r="E18" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="F18" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666702</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="22">
+        <v>45684</v>
+      </c>
+      <c r="B19" s="16"/>
+      <c r="C19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="11">
+        <v>0.374999999999999</v>
+      </c>
+      <c r="E19" s="11">
+        <v>0.54166666666666696</v>
+      </c>
+      <c r="F19" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666796</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A20" s="22">
+        <v>45685</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="11">
+        <v>0.41666666666666502</v>
+      </c>
+      <c r="E20" s="11">
+        <v>0.58333333333333304</v>
+      </c>
+      <c r="F20" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666802</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="22">
+        <v>45686</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="11">
+        <v>0.45833333333333098</v>
+      </c>
+      <c r="E21" s="11">
+        <v>0.625</v>
+      </c>
+      <c r="F21" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666902</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="22">
+        <v>45687</v>
+      </c>
+      <c r="B22" s="16"/>
+      <c r="C22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="11">
+        <v>0.499999999999998</v>
+      </c>
+      <c r="E22" s="11">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="F22" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666796</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="22">
+        <v>45688</v>
+      </c>
+      <c r="B23" s="16"/>
+      <c r="C23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="11">
+        <v>0.54166666666666397</v>
+      </c>
+      <c r="E23" s="11">
+        <v>0.70833333333333304</v>
+      </c>
+      <c r="F23" s="13">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666907</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="2"/>
       <c r="D24" s="11"/>
       <c r="E24" s="11"/>
@@ -1052,8 +1139,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="2"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
@@ -1063,8 +1150,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="2"/>
       <c r="D26" s="11"/>
       <c r="E26" s="11"/>
@@ -1074,8 +1161,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" s="7" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="2"/>
       <c r="D27" s="11"/>
       <c r="E27" s="11"/>
@@ -1091,43 +1178,43 @@
       </c>
       <c r="F29" s="14">
         <f>IF(SUM(F12:F27)=0,"",SUM(F12:F27))</f>
-        <v>0.16666666666666663</v>
+        <v>2.0000000000000089</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31" s="23">
         <v>45693</v>
       </c>
-      <c r="B31" s="16"/>
+      <c r="B31" s="24"/>
       <c r="C31" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="17"/>
+      <c r="B32" s="25"/>
       <c r="C32" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="33" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="16"/>
+      <c r="B34" s="24"/>
       <c r="C34" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B35" s="17"/>
+      <c r="B35" s="25"/>
       <c r="C35" s="8" t="s">
         <v>14</v>
       </c>
@@ -1222,6 +1309,19 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A24:B24"/>
@@ -1231,21 +1331,8 @@
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.59055118110236227" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>